<commit_message>
fix: Paddle billing bugs + annual toggle + docs update
</commit_message>
<xml_diff>
--- a/checklists/POTAL_B2B_Checklist.xlsx
+++ b/checklists/POTAL_B2B_Checklist.xlsx
@@ -805,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I154"/>
+  <dimension ref="A1:I159"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="18" min="1" max="1"/>
@@ -4317,7 +4317,7 @@
       </c>
       <c r="F75" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G75" s="25" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="I75" s="22" t="inlineStr">
         <is>
-          <t>⚠️ 구 요금제(Starter $9)로 1개 생성됨 → 삭제 후 신 요금제로 재생성 필요: Basic $20, Pro $80, Enterprise $300</t>
+          <t>세션 36-37: Basic/Pro/Enterprise × Monthly/Annual 6개 Price 생성</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G76" s="25" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="I76" s="22" t="inlineStr">
         <is>
-          <t>기존 LemonSqueezy createCheckout() → Paddle SDK로 재작성 필요</t>
+          <t>세션 36: paddle.ts + checkout/route.ts 구현 완료</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="F77" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G77" s="25" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="I77" s="22" t="inlineStr">
         <is>
-          <t>기존 LS webhook → Paddle webhook으로 재작성 필요</t>
+          <t>세션 36: webhook/route.ts Paddle Signature 검증 + 6개 이벤트</t>
         </is>
       </c>
     </row>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G78" s="25" t="inlineStr">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="I78" s="22" t="inlineStr">
         <is>
-          <t>기존 LS 상태 매핑 → Paddle 상태 매핑으로 변경 필요</t>
+          <t>세션 36: subscription.ts Paddle 상태 매핑 + cancel/pause/resume</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="I84" s="28" t="inlineStr">
         <is>
-          <t>✅ 세션 26: dashboard Logs 탭. /api/v1/sellers/analytics?type=logs API. 최근 100건 테이블</t>
+          <t>세션 37: 4-02와 동일 (중복 태스크). 6개 Price 생성 완료</t>
         </is>
       </c>
     </row>
@@ -6853,7 +6853,7 @@
       </c>
       <c r="D132" s="41" t="inlineStr">
         <is>
-          <t>DDP 체크아웃 통합 (Stripe 연동)</t>
+          <t>DDP 체크아웃 통합 (Paddle 연동)</t>
         </is>
       </c>
       <c r="E132" s="41" t="inlineStr">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="I132" s="41" t="inlineStr">
         <is>
-          <t>Pro+ 전용. Stripe Payment Intent + TLC 통합</t>
+          <t>Stripe→Paddle 전환 완료. DDP 구현은 Phase 6</t>
         </is>
       </c>
     </row>
@@ -7192,7 +7192,7 @@
       </c>
       <c r="F139" s="40" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G139" s="40" t="inlineStr">
@@ -7207,7 +7207,7 @@
       </c>
       <c r="I139" s="41" t="inlineStr">
         <is>
-          <t>구 요금제(Free500/Starter$9/Growth$29) → 신(Free100/Basic$20/Pro$80/Enterprise$300). 7개 파일. Paddle 전환 후 일괄</t>
+          <t>세션 36: plan-checker, pricing page, dashboard 등 12개 파일 업데이트</t>
         </is>
       </c>
     </row>
@@ -7494,382 +7494,663 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr">
+      <c r="A146" s="18" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
+      <c r="B146" s="18" t="inlineStr">
         <is>
           <t>프로젝트 정리</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C146" s="18" t="inlineStr">
         <is>
           <t>6-18</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr">
+      <c r="D146" s="18" t="inlineStr">
         <is>
           <t>B2C 잔재 파일/폴더 삭제 (ios/, capacitor, 등 8개)</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
+      <c r="E146" s="18" t="inlineStr">
         <is>
           <t>git branch potal-b2c-snapshot</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr">
+      <c r="F146" s="18" t="inlineStr">
         <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr">
+      <c r="G146" s="18" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr">
+      <c r="H146" s="18" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr">
+      <c r="I146" s="18" t="inlineStr">
         <is>
           <t>세션 36: B2C 백업 후 삭제. Capacitor npm uninstall은 Mac에서 별도 실행 필요</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr">
+      <c r="A147" s="18" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
+      <c r="B147" s="18" t="inlineStr">
         <is>
           <t>프로젝트 정리</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
+      <c r="C147" s="18" t="inlineStr">
         <is>
           <t>6-19</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr">
+      <c r="D147" s="18" t="inlineStr">
         <is>
           <t>중복/대체 파일 삭제 (5개)</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr">
+      <c r="E147" s="18" t="inlineStr">
         <is>
           <t>analysis/, checklists/, docs/</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr">
+      <c r="F147" s="18" t="inlineStr">
         <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr">
+      <c r="G147" s="18" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr">
+      <c r="H147" s="18" t="inlineStr">
         <is>
           <t>0.5h</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr">
+      <c r="I147" s="18" t="inlineStr">
         <is>
           <t>세션 36: v2.xlsx로 대체된 파일, 완료된 TODO, 중복 INDEX.md</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr">
+      <c r="A148" s="18" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+      <c r="B148" s="18" t="inlineStr">
         <is>
           <t>프로젝트 정리</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
+      <c r="C148" s="18" t="inlineStr">
         <is>
           <t>6-20</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr">
+      <c r="D148" s="18" t="inlineStr">
         <is>
           <t>파일 이동/구조 정리 (tariff-research, archive)</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr">
+      <c r="E148" s="18" t="inlineStr">
         <is>
           <t>data/tariff-research/, archive/</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr">
+      <c r="F148" s="18" t="inlineStr">
         <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr">
+      <c r="G148" s="18" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr">
+      <c r="H148" s="18" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr">
+      <c r="I148" s="18" t="inlineStr">
         <is>
           <t>세션 36: data/ 루트→tariff-research/ 14개, archive/ 3개, .DS_Store 7개 삭제</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
+      <c r="A149" s="18" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B149" s="18" t="inlineStr">
         <is>
           <t>프로젝트 정리</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C149" s="18" t="inlineStr">
         <is>
           <t>6-21</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr">
+      <c r="D149" s="18" t="inlineStr">
         <is>
           <t>요금제 구/신 불일치 검증 + 문서 반영</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr">
+      <c r="E149" s="18" t="inlineStr">
         <is>
           <t>session-context.md, CLAUDE.md 등</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr">
+      <c r="F149" s="18" t="inlineStr">
         <is>
           <t>✅ Done</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr">
+      <c r="G149" s="18" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr">
+      <c r="H149" s="18" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr">
+      <c r="I149" s="18" t="inlineStr">
         <is>
           <t>세션 36: 세션 28 요금제 변경 추적, Paddle Sandbox 구 요금제 확인, 5개 문서 업데이트</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr">
+      <c r="A150" s="18" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B150" s="18" t="inlineStr">
         <is>
           <t>프로젝트 정리</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
+      <c r="C150" s="18" t="inlineStr">
         <is>
           <t>6-22</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr">
+      <c r="D150" s="18" t="inlineStr">
         <is>
           <t>Capacitor 패키지 7개 npm uninstall</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr">
+      <c r="E150" s="18" t="inlineStr">
         <is>
           <t>package.json</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr">
+      <c r="F150" s="18" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr">
+      <c r="G150" s="18" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr">
+      <c r="H150" s="18" t="inlineStr">
         <is>
           <t>0.5h</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr">
+      <c r="I150" s="18" t="inlineStr">
         <is>
           <t>Mac에서 실행: npm uninstall @capacitor/app browser cli core ios splash-screen status-bar</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
+      <c r="A151" s="18" t="inlineStr">
         <is>
           <t>Phase 4</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B151" s="18" t="inlineStr">
         <is>
           <t>결제 시스템</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C151" s="18" t="inlineStr">
         <is>
           <t>4-11</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr">
+      <c r="D151" s="18" t="inlineStr">
         <is>
           <t>Paddle Sandbox 제품 재생성 (신 요금제)</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
+      <c r="E151" s="18" t="inlineStr">
         <is>
           <t>Paddle Dashboard</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr">
+      <c r="F151" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G151" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H151" s="18" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="I151" s="18" t="inlineStr">
+        <is>
+          <t>세션 37: 4-02와 동일 (중복 태스크). 6개 Price 생성 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="18" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>결제 시스템</t>
+        </is>
+      </c>
+      <c r="C152" s="18" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+      <c r="D152" s="18" t="inlineStr">
+        <is>
+          <t>Paddle API Key + Webhook 설정</t>
+        </is>
+      </c>
+      <c r="E152" s="18" t="inlineStr">
+        <is>
+          <t>Paddle Dashboard + .env</t>
+        </is>
+      </c>
+      <c r="F152" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G152" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H152" s="18" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="I152" s="18" t="inlineStr">
+        <is>
+          <t>세션 37: .env.local + Vercel 환경변수 9개 자동 추가 (API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="18" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t>결제 시스템</t>
+        </is>
+      </c>
+      <c r="C153" s="18" t="inlineStr">
+        <is>
+          <t>4-13</t>
+        </is>
+      </c>
+      <c r="D153" s="18" t="inlineStr">
+        <is>
+          <t>LemonSqueezy → Paddle SDK 전환 (코드)</t>
+        </is>
+      </c>
+      <c r="E153" s="18" t="inlineStr">
+        <is>
+          <t>app/api/billing/</t>
+        </is>
+      </c>
+      <c r="F153" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G153" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H153" s="18" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I153" s="18" t="inlineStr">
+        <is>
+          <t>세션 36: paddle.ts 신규, checkout/webhook/portal/subscription 전환</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>결제</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>4-14</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Paddle 프로덕션 전환 (Sandbox→Live API Key)</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>.env.local, Vercel</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr">
+      <c r="G154" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr">
+      <c r="H154" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr">
-        <is>
-          <t>구 Starter $9 삭제 → Basic $20, Pro $80, Enterprise $300 생성</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Sandbox 테스트 완료 후 Live 키로 전환</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
         <is>
           <t>Phase 4</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>결제 시스템</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>4-12</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>Paddle API Key + Webhook 설정</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Paddle Dashboard + .env</t>
-        </is>
-      </c>
-      <c r="F152" t="inlineStr">
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>결제</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>4-15</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Annual/Overage 빌링 구현 (Paddle One-time charge API)</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>app/lib/billing/</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Overage: Basic $0.015, Pro $0.012, Enterprise $0.01/건</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>결제</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>4-16</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Paddle Customer Portal 연동 (구독 관리 UI)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>app/dashboard/</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>4-10과 통합. management_urls API</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>정리</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>6-23</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>lemonsqueezy.ts 삭제 + npm uninstall</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>app/lib/billing/</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>paddle.ts로 완전 전환 후 삭제</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>정리</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>6-24</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>i18n translations 구버전 키 정리</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>messages/</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>Sandbox에서 API key 발급, webhook URL 설정, 테스트</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>결제 시스템</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>4-13</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>LemonSqueezy → Paddle SDK 전환 (코드)</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>app/api/billing/</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr">
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>pricing.starter→pricing.free, pricing.growth→pricing.basic 등</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>정리</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>6-25</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Vercel B2C 환경변수 정리 (RapidAPI 등)</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Vercel Dashboard</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>4h</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>checkout/webhook/portal 라우트 전부 Paddle SDK로 재작성</t>
-        </is>
-      </c>
-    </row>
-    <row r="154"/>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>백업 완료: archive/vercel_env_backup_2026-03-10.txt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I98"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -8010,13 +8291,13 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: session 37 documentation update — overage billing, checklist, cross-verification
</commit_message>
<xml_diff>
--- a/checklists/POTAL_B2B_Checklist.xlsx
+++ b/checklists/POTAL_B2B_Checklist.xlsx
@@ -1238,7 +1238,7 @@
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>Starter 5K, Growth 25K, Enterprise 무제한. plan-checker.ts</t>
+          <t>세션 37: Free 100/Basic 2K/Pro 10K/Enterprise 50K. 유료 overage 허용 (Free만 hard-block). plan-checker.ts</t>
         </is>
       </c>
     </row>
@@ -6294,7 +6294,7 @@
       </c>
       <c r="I117" s="18" t="inlineStr">
         <is>
-          <t>세션 36: ~86.3M/130M행 (44개국 완료, 9개국 남음: SGP~VNM). Cowork VM에서 import_min_remaining.py</t>
+          <t>세션 36: ~92.3M/130M행 (44개국 완료, 9개국 남음: SGP~VNM). WDC 완료 후 Mac에서 진행</t>
         </is>
       </c>
     </row>
@@ -6439,7 +6439,6 @@
         </is>
       </c>
     </row>
-    <row r="121"/>
     <row r="122">
       <c r="A122" s="39" t="inlineStr">
         <is>
@@ -6458,7 +6457,6 @@
       <c r="H122" s="39" t="n"/>
       <c r="I122" s="39" t="n"/>
     </row>
-    <row r="123"/>
     <row r="124">
       <c r="A124" s="40" t="inlineStr">
         <is>
@@ -7709,7 +7707,7 @@
       </c>
       <c r="F150" s="18" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>✅ Done</t>
         </is>
       </c>
       <c r="G150" s="18" t="inlineStr">
@@ -7724,7 +7722,7 @@
       </c>
       <c r="I150" s="18" t="inlineStr">
         <is>
-          <t>Mac에서 실행: npm uninstall @capacitor/app browser cli core ios splash-screen status-bar</t>
+          <t>세션 37(Cowork3): npm uninstall 완료 + native-auth.ts stub 교체</t>
         </is>
       </c>
     </row>
@@ -7870,284 +7868,284 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
+      <c r="A154" s="18" t="inlineStr">
         <is>
           <t>Phase 4</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="18" t="inlineStr">
         <is>
           <t>결제</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C154" s="18" t="inlineStr">
         <is>
           <t>4-14</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr">
+      <c r="D154" s="18" t="inlineStr">
         <is>
           <t>Paddle 프로덕션 전환 (Sandbox→Live API Key)</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr">
+      <c r="E154" s="18" t="inlineStr">
         <is>
           <t>.env.local, Vercel</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F154" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G154" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H154" s="18" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="I154" s="18" t="inlineStr">
+        <is>
+          <t>세션 37(Cowork3): Live API Key + 6개 Live Price + Webhook 56 events. Vercel 배포 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="18" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B155" s="18" t="inlineStr">
+        <is>
+          <t>결제</t>
+        </is>
+      </c>
+      <c r="C155" s="18" t="inlineStr">
+        <is>
+          <t>4-15</t>
+        </is>
+      </c>
+      <c r="D155" s="18" t="inlineStr">
+        <is>
+          <t>Annual/Overage 빌링 구현 (Paddle One-time charge API)</t>
+        </is>
+      </c>
+      <c r="E155" s="18" t="inlineStr">
+        <is>
+          <t>app/lib/billing/</t>
+        </is>
+      </c>
+      <c r="F155" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G155" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H155" s="18" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I155" s="18" t="inlineStr">
+        <is>
+          <t>세션 37(Cowork3): overage.ts + billing-overage cron + plan-checker overage 허용 + middleware 헤더</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="18" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B156" s="18" t="inlineStr">
+        <is>
+          <t>결제</t>
+        </is>
+      </c>
+      <c r="C156" s="18" t="inlineStr">
+        <is>
+          <t>4-16</t>
+        </is>
+      </c>
+      <c r="D156" s="18" t="inlineStr">
+        <is>
+          <t>Paddle Customer Portal 연동 (구독 관리 UI)</t>
+        </is>
+      </c>
+      <c r="E156" s="18" t="inlineStr">
+        <is>
+          <t>app/dashboard/</t>
+        </is>
+      </c>
+      <c r="F156" s="18" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
+      <c r="G156" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H156" s="18" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="I156" s="18" t="inlineStr">
+        <is>
+          <t>4-10과 통합. management_urls API</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="18" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B157" s="18" t="inlineStr">
+        <is>
+          <t>정리</t>
+        </is>
+      </c>
+      <c r="C157" s="18" t="inlineStr">
+        <is>
+          <t>6-23</t>
+        </is>
+      </c>
+      <c r="D157" s="18" t="inlineStr">
+        <is>
+          <t>lemonsqueezy.ts 삭제 + npm uninstall</t>
+        </is>
+      </c>
+      <c r="E157" s="18" t="inlineStr">
+        <is>
+          <t>app/lib/billing/</t>
+        </is>
+      </c>
+      <c r="F157" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G157" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H157" s="18" t="inlineStr">
+        <is>
+          <t>0.5h</t>
+        </is>
+      </c>
+      <c r="I157" s="18" t="inlineStr">
+        <is>
+          <t>세션 37(Cowork3): lemonsqueezy.ts 삭제 + npm uninstall @lemonsqueezy/lemonsqueezy.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="18" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B158" s="18" t="inlineStr">
+        <is>
+          <t>정리</t>
+        </is>
+      </c>
+      <c r="C158" s="18" t="inlineStr">
+        <is>
+          <t>6-24</t>
+        </is>
+      </c>
+      <c r="D158" s="18" t="inlineStr">
+        <is>
+          <t>i18n translations 구버전 키 정리</t>
+        </is>
+      </c>
+      <c r="E158" s="18" t="inlineStr">
+        <is>
+          <t>messages/</t>
+        </is>
+      </c>
+      <c r="F158" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G158" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H158" s="18" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>Sandbox 테스트 완료 후 Live 키로 전환</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>결제</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>4-15</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>Annual/Overage 빌링 구현 (Paddle One-time charge API)</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>app/lib/billing/</t>
-        </is>
-      </c>
-      <c r="F155" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>4h</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>Overage: Basic $0.015, Pro $0.012, Enterprise $0.01/건</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>결제</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>4-16</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>Paddle Customer Portal 연동 (구독 관리 UI)</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>app/dashboard/</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>3h</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>4-10과 통합. management_urls API</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
+      <c r="I158" s="18" t="inlineStr">
+        <is>
+          <t>세션 37(Cowork3): 6개 언어 키 전면 교체 (starter→free, growth→basic+pro, scale→enterprise, annual 추가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="18" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B159" s="18" t="inlineStr">
         <is>
           <t>정리</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>6-23</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>lemonsqueezy.ts 삭제 + npm uninstall</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>app/lib/billing/</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G157" t="inlineStr">
+      <c r="C159" s="18" t="inlineStr">
+        <is>
+          <t>6-25</t>
+        </is>
+      </c>
+      <c r="D159" s="18" t="inlineStr">
+        <is>
+          <t>Vercel B2C 환경변수 정리 (RapidAPI 등)</t>
+        </is>
+      </c>
+      <c r="E159" s="18" t="inlineStr">
+        <is>
+          <t>Vercel Dashboard</t>
+        </is>
+      </c>
+      <c r="F159" s="18" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G159" s="18" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr">
+      <c r="H159" s="18" t="inlineStr">
         <is>
           <t>0.5h</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>paddle.ts로 완전 전환 후 삭제</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>정리</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>6-24</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>i18n translations 구버전 키 정리</t>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>messages/</t>
-        </is>
-      </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>1h</t>
-        </is>
-      </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>pricing.starter→pricing.free, pricing.growth→pricing.basic 등</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>정리</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>6-25</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>Vercel B2C 환경변수 정리 (RapidAPI 등)</t>
-        </is>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>Vercel Dashboard</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>0.5h</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>백업 완료: archive/vercel_env_backup_2026-03-10.txt</t>
+      <c r="I159" s="18" t="inlineStr">
+        <is>
+          <t>세션 37(Cowork3): 15개 삭제 (ALIEXPRESS/AMAZON/EBAY/RAPIDAPI/APIFY/TEMU). 36→21개</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CW7: Chief Orchestrator 운영 체계 확정 (15 Division + 3 Layer)
- POTAL_AI_Agent_Org.html v3 완성 (일일 운영 플로우 5단계 리디자인)
- CLAUDE.md에 Chief Orchestrator 프로토콜 전체 반영
- session-context.md, .cursorrules, CHANGELOG.md 업데이트
- POTAL_B2B_Checklist.xlsx CW7 태스크 10건 추가
- NEXT_SESSION_START.md 전면 재작성
- SESSION_CW7_REPORT.md 세션 리포트 생성
</commit_message>
<xml_diff>
--- a/checklists/POTAL_B2B_Checklist.xlsx
+++ b/checklists/POTAL_B2B_Checklist.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -146,8 +146,12 @@
     <font>
       <color rgb="00FF8C00"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -228,6 +232,16 @@
         <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -277,7 +291,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -423,6 +437,12 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -805,7 +825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I159"/>
+  <dimension ref="A1:I169"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="18" min="1" max="1"/>
@@ -8146,6 +8166,476 @@
       <c r="I159" s="18" t="inlineStr">
         <is>
           <t>세션 37(Cowork3): 15개 삭제 (ALIEXPRESS/AMAZON/EBAY/RAPIDAPI/APIFY/TEMU). 36→21개</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="53" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B160" s="53" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C160" s="53" t="inlineStr">
+        <is>
+          <t>CW7-01</t>
+        </is>
+      </c>
+      <c r="D160" s="53" t="inlineStr">
+        <is>
+          <t>AI Agent Org v2→v3 재설계 (10→15 Division, 3 Layer)</t>
+        </is>
+      </c>
+      <c r="E160" s="53" t="inlineStr">
+        <is>
+          <t>POTAL_AI_Agent_Org.html</t>
+        </is>
+      </c>
+      <c r="F160" s="53" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G160" s="53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H160" s="53" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="I160" s="53" t="inlineStr">
+        <is>
+          <t>15 Division + Automation/Monitor/Active Layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="53" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B161" s="53" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C161" s="53" t="inlineStr">
+        <is>
+          <t>CW7-02</t>
+        </is>
+      </c>
+      <c r="D161" s="53" t="inlineStr">
+        <is>
+          <t>CLAUDE.md Chief Orchestrator 운영 프로토콜 반영</t>
+        </is>
+      </c>
+      <c r="E161" s="53" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="F161" s="53" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G161" s="53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H161" s="53" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="I161" s="53" t="inlineStr">
+        <is>
+          <t>역할정의, 15 Division 테이블, Morning Brief, Layer 모델, Escalation Flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="53" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B162" s="53" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C162" s="53" t="inlineStr">
+        <is>
+          <t>CW7-03</t>
+        </is>
+      </c>
+      <c r="D162" s="53" t="inlineStr">
+        <is>
+          <t>일일 운영 플로우 v3 상세화 (Phase 0~4 + 주간/월간)</t>
+        </is>
+      </c>
+      <c r="E162" s="53" t="inlineStr">
+        <is>
+          <t>POTAL_AI_Agent_Org.html</t>
+        </is>
+      </c>
+      <c r="F162" s="53" t="inlineStr">
+        <is>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="G162" s="53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H162" s="53" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="I162" s="53" t="inlineStr">
+        <is>
+          <t>Phase 0 자동~Phase 4 마감, 주간 월/월간 1일 루틴</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="54" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B163" s="54" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C163" s="54" t="inlineStr">
+        <is>
+          <t>CW7-04</t>
+        </is>
+      </c>
+      <c r="D163" s="54" t="inlineStr">
+        <is>
+          <t>Division Layer 1 자동화 세팅 — D8 QA 자동 스팟체크</t>
+        </is>
+      </c>
+      <c r="E163" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F163" s="54" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G163" s="54" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H163" s="54" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I163" s="54" t="inlineStr">
+        <is>
+          <t>D8 ❌ 미구현. CI 테스트만 있음</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="54" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B164" s="54" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C164" s="54" t="inlineStr">
+        <is>
+          <t>CW7-05</t>
+        </is>
+      </c>
+      <c r="D164" s="54" t="inlineStr">
+        <is>
+          <t>Division Layer 1 자동화 세팅 — D9 Customer Success</t>
+        </is>
+      </c>
+      <c r="E164" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F164" s="54" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G164" s="54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H164" s="54" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="I164" s="54" t="inlineStr">
+        <is>
+          <t>D9 ❌ 미구현. 챗봇/온보딩 자동화 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="54" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B165" s="54" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C165" s="54" t="inlineStr">
+        <is>
+          <t>CW7-06</t>
+        </is>
+      </c>
+      <c r="D165" s="54" t="inlineStr">
+        <is>
+          <t>Division Layer 1 자동화 세팅 — D11 에러 모니터링</t>
+        </is>
+      </c>
+      <c r="E165" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F165" s="54" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G165" s="54" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H165" s="54" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="I165" s="54" t="inlineStr">
+        <is>
+          <t>D11 ⚠️ 부분. 에러 모니터링/알림 미구현</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="54" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B166" s="54" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C166" s="54" t="inlineStr">
+        <is>
+          <t>CW7-07</t>
+        </is>
+      </c>
+      <c r="D166" s="54" t="inlineStr">
+        <is>
+          <t>Division Layer 1 자동화 세팅 — D12 Make.com 마케팅</t>
+        </is>
+      </c>
+      <c r="E166" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F166" s="54" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G166" s="54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H166" s="54" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="I166" s="54" t="inlineStr">
+        <is>
+          <t>D12 ❌ 미구현. Make.com 포스팅/이메일 미설정</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="54" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B167" s="54" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C167" s="54" t="inlineStr">
+        <is>
+          <t>CW7-08</t>
+        </is>
+      </c>
+      <c r="D167" s="54" t="inlineStr">
+        <is>
+          <t>Division Layer 1 자동화 세팅 — D14 비용 데이터 수집</t>
+        </is>
+      </c>
+      <c r="E167" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F167" s="54" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G167" s="54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H167" s="54" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="I167" s="54" t="inlineStr">
+        <is>
+          <t>D14 ❌ 미구현. 비용 데이터 자동 수집 미설정</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="54" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B168" s="54" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C168" s="54" t="inlineStr">
+        <is>
+          <t>CW7-09</t>
+        </is>
+      </c>
+      <c r="D168" s="54" t="inlineStr">
+        <is>
+          <t>Division Layer 1 자동화 세팅 — D15 RSS/뉴스 수집</t>
+        </is>
+      </c>
+      <c r="E168" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F168" s="54" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G168" s="54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H168" s="54" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="I168" s="54" t="inlineStr">
+        <is>
+          <t>D15 ❌ 미구현. RSS/뉴스 자동 수집 미설정</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="54" t="inlineStr">
+        <is>
+          <t>CW7</t>
+        </is>
+      </c>
+      <c r="B169" s="54" t="inlineStr">
+        <is>
+          <t>AI Operations</t>
+        </is>
+      </c>
+      <c r="C169" s="54" t="inlineStr">
+        <is>
+          <t>CW7-10</t>
+        </is>
+      </c>
+      <c r="D169" s="54" t="inlineStr">
+        <is>
+          <t>Division Layer 1 자동화 세팅 — D13 캘린더 알림</t>
+        </is>
+      </c>
+      <c r="E169" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F169" s="54" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="G169" s="54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H169" s="54" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="I169" s="54" t="inlineStr">
+        <is>
+          <t>D13 ❌ 미구현. 계약 만료 캘린더 알림 미설정</t>
         </is>
       </c>
     </row>

</xml_diff>